<commit_message>
Hybrid Framework Design Day-5
</commit_message>
<xml_diff>
--- a/TestData/Data.xlsx
+++ b/TestData/Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Trainings\SA_Automation_2025_2\HybridFramework\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51623C06-9A80-4223-8538-A18128C50AB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A53A02F1-C46F-4053-8179-2090599C0921}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>standard_user</t>
   </si>
@@ -52,6 +52,9 @@
   </si>
   <si>
     <t>pc</t>
+  </si>
+  <si>
+    <t>"411047"</t>
   </si>
 </sst>
 </file>
@@ -456,8 +459,8 @@
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="1">
-        <v>411047</v>
+      <c r="B5" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>